<commit_message>
feat: update contact details across the application with new business phone number
</commit_message>
<xml_diff>
--- a/docs/client/Xhosen-Gate-Offer-and-Price-Review.xlsx
+++ b/docs/client/Xhosen-Gate-Offer-and-Price-Review.xlsx
@@ -120,7 +120,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -142,11 +142,55 @@
         <color rgb="00DCD5C9"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DCD5C9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DCD5C9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DCD5C9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00DCD5C9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DCD5C9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00DCD5C9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00DCD5C9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00DCD5C9"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -200,6 +244,8 @@
       <alignment horizontal="right" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -591,6 +637,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="46" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -651,6 +698,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -692,6 +740,9 @@
           <t>Airport and city-to-city transfer prices (the quote widget on the home page)</t>
         </is>
       </c>
+      <c r="D12" s="21" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
@@ -707,6 +758,9 @@
           <t>Every vehicle and its starting price</t>
         </is>
       </c>
+      <c r="D13" s="21" t="n"/>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="22" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
@@ -722,6 +776,9 @@
           <t>Multi-day tours from Marrakech</t>
         </is>
       </c>
+      <c r="D14" s="21" t="n"/>
+      <c r="E14" s="21" t="n"/>
+      <c r="F14" s="22" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -737,6 +794,9 @@
           <t>One and two-day excursions</t>
         </is>
       </c>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="22" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
@@ -752,6 +812,9 @@
           <t>Cooking class, quad, camel, food tour, balloon</t>
         </is>
       </c>
+      <c r="D16" s="21" t="n"/>
+      <c r="E16" s="21" t="n"/>
+      <c r="F16" s="22" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -767,6 +830,9 @@
           <t>Airport transfer, hotel transfer, car with driver</t>
         </is>
       </c>
+      <c r="D17" s="21" t="n"/>
+      <c r="E17" s="21" t="n"/>
+      <c r="F17" s="22" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -833,6 +899,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -1043,6 +1110,7 @@
       <c r="G10" s="12" t="n"/>
       <c r="H10" s="13" t="n"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
@@ -1099,6 +1167,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -1333,6 +1402,7 @@
       <c r="G12" s="12" t="n"/>
       <c r="H12" s="13" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
@@ -1392,6 +1462,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -1705,6 +1776,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -2120,6 +2192,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -2417,6 +2490,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -2623,6 +2697,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -2653,7 +2728,7 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>+212 672 958 587</t>
+          <t>+212 663 227 698</t>
         </is>
       </c>
       <c r="C5" s="11" t="n"/>
@@ -2667,7 +2742,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>+212672958587</t>
+          <t>+212663227698</t>
         </is>
       </c>
       <c r="C6" s="11" t="n"/>
@@ -2681,7 +2756,7 @@
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>+212 672 958 587  ·  wa.me/212672958587</t>
+          <t>+212 663 227 698  ·  wa.me/212663227698</t>
         </is>
       </c>
       <c r="C7" s="11" t="n"/>
@@ -2785,6 +2860,7 @@
       <c r="C14" s="11" t="n"/>
       <c r="D14" s="13" t="n"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="20" t="inlineStr">
         <is>
@@ -2798,6 +2874,9 @@
           <t>• The address above is a placeholder — the real street address is needed for the contact page and for Google.</t>
         </is>
       </c>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="21" t="n"/>
+      <c r="D17" s="22" t="n"/>
     </row>
     <row r="18" ht="34" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -2805,6 +2884,9 @@
           <t>• The Google rating, review count and Maps link are placeholders. Displaying a rating you have not earned is a real risk: we need your Google Business Profile link and its true numbers, or we remove the rating block.</t>
         </is>
       </c>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="21" t="n"/>
+      <c r="D18" s="22" t="n"/>
     </row>
     <row r="19" ht="34" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
@@ -2812,13 +2894,19 @@
           <t>• Customer reviews shown on the tour, excursion and activity pages are sample text. Send real ones, or we take them down.</t>
         </is>
       </c>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="21" t="n"/>
+      <c r="D19" s="22" t="n"/>
     </row>
     <row r="20" ht="34" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>• Every WhatsApp button now points at +212 672 958 587. Confirm this is the phone that should receive bookings.</t>
-        </is>
-      </c>
+          <t>• Every WhatsApp button now points at +212 663 227 698. Confirm this is the phone that should receive bookings.</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="21" t="n"/>
+      <c r="D20" s="22" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2865,6 +2953,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
@@ -3048,7 +3137,7 @@
       </c>
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>Confirm +212 672 958 587 is the booking WhatsApp and phone</t>
+          <t>Confirm +212 663 227 698 is the booking WhatsApp and phone</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">

</xml_diff>